<commit_message>
Record Zenodo DOIs for v1.0.4, run outputs and library metadata; update Table 13 workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015yTwpiqdsKGArv5WSRMqT6
</commit_message>
<xml_diff>
--- a/supplement/handcurated/Supplementary_Table_13_Sequencing_library_inventory_and_quality_metrics.xlsx
+++ b/supplement/handcurated/Supplementary_Table_13_Sequencing_library_inventory_and_quality_metrics.xlsx
@@ -10695,7 +10695,7 @@
       </c>
       <c r="AL37" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM37" s="9" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="AL38" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM38" s="9" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="AL39" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM39" s="9" t="inlineStr">
@@ -11509,7 +11509,7 @@
       </c>
       <c r="AL40" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM40" s="9" t="inlineStr">
@@ -11779,7 +11779,7 @@
       </c>
       <c r="AL41" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM41" s="9" t="inlineStr">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="AL42" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM42" s="9" t="inlineStr">
@@ -12319,7 +12319,7 @@
       </c>
       <c r="AL43" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM43" s="9" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="AL44" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM44" s="9" t="inlineStr">
@@ -12859,7 +12859,7 @@
       </c>
       <c r="AL45" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM45" s="9" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="AL46" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM46" s="9" t="inlineStr">
@@ -13399,7 +13399,7 @@
       </c>
       <c r="AL47" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM47" s="9" t="inlineStr">
@@ -13669,7 +13669,7 @@
       </c>
       <c r="AL48" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM48" s="9" t="inlineStr">
@@ -13939,7 +13939,7 @@
       </c>
       <c r="AL49" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM49" s="9" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="AL50" s="9" t="inlineStr">
         <is>
-          <t>trigeminal pilot (Supp. Table 12)</t>
+          <t>trigeminal pilot (Supplementary Table 12)</t>
         </is>
       </c>
       <c r="AM50" s="9" t="inlineStr">

</xml_diff>